<commit_message>
test(wallet): WALLET-PHONE-01.2 evidence tail — partner-ready PNGs and strict BFF/XLSX
Wait for loaded partner rows before visual-01-2 captures; validate export scope via
partners + groupKey orders (HTTP 200) and XLSX eachRow parity; pin codeUnderTest a8f6947.

Co-authored-by: kraavediks <kraavediks@gmail.com>
</commit_message>
<xml_diff>
--- a/artifacts/remcard-wallet-phone/smoke-export-01-2.xlsx
+++ b/artifacts/remcard-wallet-phone/smoke-export-01-2.xlsx
@@ -26,13 +26,13 @@
     <t>Область выгрузки</t>
   </si>
   <si>
-    <t>Обзор · Мне должны</t>
+    <t>Партнёры · текущий отбор</t>
   </si>
   <si>
     <t>Выгружено (UTC)</t>
   </si>
   <si>
-    <t>2026-10-17T05:19:22.762Z</t>
+    <t>2026-10-17T05:23:42.791Z</t>
   </si>
   <si>
     <t>Часовой пояс дат в листах</t>
@@ -203,7 +203,7 @@
     <t>Статус детализации</t>
   </si>
   <si>
-    <t>cmvby5g2j004fjs9gihfypp5h</t>
+    <t>cmvbyb0bb004fjs9vzhijnfql</t>
   </si>
   <si>
     <t/>
@@ -215,10 +215,10 @@
     <t>Исторические реквизиты не сохранены</t>
   </si>
   <si>
-    <t>GBR7Y34T</t>
-  </si>
-  <si>
-    <t>RC-R05B-1792214351436-2</t>
+    <t>LC03KGBT</t>
+  </si>
+  <si>
+    <t>RC-R05B-1792214610960-2</t>
   </si>
   <si>
     <t>Не согласован</t>
@@ -230,181 +230,181 @@
     <t>Строки заказа загружены</t>
   </si>
   <si>
-    <t>cmvby5g2h004ajs9g8h7w9jkf</t>
-  </si>
-  <si>
-    <t>J6G0JWF5</t>
-  </si>
-  <si>
-    <t>RC-R05-1792214351421-1</t>
-  </si>
-  <si>
-    <t>cmvby5g2f0045js9gyqij1sg5</t>
-  </si>
-  <si>
-    <t>4ZQ8OIE0</t>
-  </si>
-  <si>
-    <t>cmvby5g2d0040js9gjwxi8c2r</t>
-  </si>
-  <si>
-    <t>IYFKYPPC</t>
-  </si>
-  <si>
-    <t>cmvby5g2b003vjs9g6gaxnxa6</t>
-  </si>
-  <si>
-    <t>RUVUM57V</t>
-  </si>
-  <si>
-    <t>cmvby5g29003qjs9gqyq2x88x</t>
-  </si>
-  <si>
-    <t>I91HV26O</t>
-  </si>
-  <si>
-    <t>cmvby5g27003ljs9guv134u8d</t>
-  </si>
-  <si>
-    <t>C003X63K</t>
-  </si>
-  <si>
-    <t>cmvby5g24003gjs9gqpumcpev</t>
-  </si>
-  <si>
-    <t>NRIM4DDM</t>
-  </si>
-  <si>
-    <t>cmvby5g21003bjs9gy3mri2kn</t>
-  </si>
-  <si>
-    <t>AZI2FFWR</t>
-  </si>
-  <si>
-    <t>cmvby5g1z0036js9gtanqvxx5</t>
-  </si>
-  <si>
-    <t>VYLLQWJA</t>
-  </si>
-  <si>
-    <t>cmvby5g1x0031js9gy5w17kmx</t>
-  </si>
-  <si>
-    <t>GSKKPBV4</t>
-  </si>
-  <si>
-    <t>cmvby5g1v002wjs9gb3hnoyqg</t>
-  </si>
-  <si>
-    <t>DD9J27OC</t>
-  </si>
-  <si>
-    <t>cmvby5g1r002rjs9gmucbbqi2</t>
-  </si>
-  <si>
-    <t>S8DTRBN4</t>
-  </si>
-  <si>
-    <t>cmvby5g1p002mjs9g09kvzr3q</t>
-  </si>
-  <si>
-    <t>YO4KSY06</t>
-  </si>
-  <si>
-    <t>cmvby5g1n002hjs9g7ee457ba</t>
-  </si>
-  <si>
-    <t>BYDP2289</t>
-  </si>
-  <si>
-    <t>cmvby5g1l002cjs9gbfjc09ji</t>
-  </si>
-  <si>
-    <t>IV7DLN0W</t>
-  </si>
-  <si>
-    <t>cmvby5g1i0027js9gj6okgjp5</t>
-  </si>
-  <si>
-    <t>ZQY7E814</t>
-  </si>
-  <si>
-    <t>cmvby5g1g0022js9g7vw8ot2v</t>
-  </si>
-  <si>
-    <t>ZYFJTVPO</t>
-  </si>
-  <si>
-    <t>cmvby5g1d001xjs9gkqpn9hz7</t>
-  </si>
-  <si>
-    <t>3IOQURHF</t>
-  </si>
-  <si>
-    <t>cmvby5g1b001sjs9gorxbnwj2</t>
-  </si>
-  <si>
-    <t>S1F6OCFW</t>
-  </si>
-  <si>
-    <t>cmvby5g19001njs9gox6edg8i</t>
-  </si>
-  <si>
-    <t>N585F69R</t>
-  </si>
-  <si>
-    <t>cmvby5g17001ijs9gpo8jc8c4</t>
-  </si>
-  <si>
-    <t>E1OCDFGB</t>
-  </si>
-  <si>
-    <t>cmvby5g15001djs9gew40k1jn</t>
-  </si>
-  <si>
-    <t>CSDAHVHL</t>
-  </si>
-  <si>
-    <t>cmvby5g130018js9gmi4z8x63</t>
-  </si>
-  <si>
-    <t>HP4EJQWH</t>
-  </si>
-  <si>
-    <t>cmvby5g110013js9gxr573oc7</t>
-  </si>
-  <si>
-    <t>34HOU3GN</t>
-  </si>
-  <si>
-    <t>cmvby5g0y000yjs9gucu7s91g</t>
-  </si>
-  <si>
-    <t>P0NPJ3Q7</t>
-  </si>
-  <si>
-    <t>cmvby5g0w000tjs9g8g56gea1</t>
-  </si>
-  <si>
-    <t>0O7ANACO</t>
-  </si>
-  <si>
-    <t>cmvby5g0u000ojs9gntd4yyka</t>
-  </si>
-  <si>
-    <t>WUBJHWHV</t>
-  </si>
-  <si>
-    <t>cmvby5g0r000jjs9gq5q4iaji</t>
-  </si>
-  <si>
-    <t>LZ574148</t>
-  </si>
-  <si>
-    <t>cmvby5g0o000ejs9gsm33fatw</t>
-  </si>
-  <si>
-    <t>A6OEZ1T0</t>
+    <t>cmvbyb0b9004ajs9v747ovoa2</t>
+  </si>
+  <si>
+    <t>LKDXM8OW</t>
+  </si>
+  <si>
+    <t>RC-R05-1792214610949-1</t>
+  </si>
+  <si>
+    <t>cmvbyb0b70045js9vin9jvqgq</t>
+  </si>
+  <si>
+    <t>CJBRHPFJ</t>
+  </si>
+  <si>
+    <t>cmvbyb0b50040js9vgegr1tc8</t>
+  </si>
+  <si>
+    <t>QIUZEZGG</t>
+  </si>
+  <si>
+    <t>cmvbyb0b4003vjs9vuofvnh0t</t>
+  </si>
+  <si>
+    <t>BHCM05EK</t>
+  </si>
+  <si>
+    <t>cmvbyb0b2003qjs9v0px1antl</t>
+  </si>
+  <si>
+    <t>P9M18FT2</t>
+  </si>
+  <si>
+    <t>cmvbyb0b0003ljs9viruw23lc</t>
+  </si>
+  <si>
+    <t>6C6GL77T</t>
+  </si>
+  <si>
+    <t>cmvbyb0ay003gjs9v3dyubuhq</t>
+  </si>
+  <si>
+    <t>47CWR076</t>
+  </si>
+  <si>
+    <t>cmvbyb0aw003bjs9vck3yqhjp</t>
+  </si>
+  <si>
+    <t>U92YKAVK</t>
+  </si>
+  <si>
+    <t>cmvbyb0au0036js9v8hgkbgm0</t>
+  </si>
+  <si>
+    <t>UUS4995X</t>
+  </si>
+  <si>
+    <t>cmvbyb0as0031js9vtxry8a7e</t>
+  </si>
+  <si>
+    <t>VD41ZA8K</t>
+  </si>
+  <si>
+    <t>cmvbyb0aq002wjs9vdcysoxhi</t>
+  </si>
+  <si>
+    <t>0L45ACG7</t>
+  </si>
+  <si>
+    <t>cmvbyb0an002rjs9v3jc0nbhz</t>
+  </si>
+  <si>
+    <t>SV8U2SA1</t>
+  </si>
+  <si>
+    <t>cmvbyb0am002mjs9vcwdp2mxh</t>
+  </si>
+  <si>
+    <t>0IVHRG2H</t>
+  </si>
+  <si>
+    <t>cmvbyb0ak002hjs9voyhaud1p</t>
+  </si>
+  <si>
+    <t>17US3XJU</t>
+  </si>
+  <si>
+    <t>cmvbyb0ai002cjs9vcnkhbn7v</t>
+  </si>
+  <si>
+    <t>CMUYO8II</t>
+  </si>
+  <si>
+    <t>cmvbyb0af0027js9vh71uk27y</t>
+  </si>
+  <si>
+    <t>UIV2JDSD</t>
+  </si>
+  <si>
+    <t>cmvbyb0ad0022js9vrwgutzk4</t>
+  </si>
+  <si>
+    <t>DOL9HIV8</t>
+  </si>
+  <si>
+    <t>cmvbyb0ac001xjs9veqf49dn8</t>
+  </si>
+  <si>
+    <t>1ABWOUQS</t>
+  </si>
+  <si>
+    <t>cmvbyb0aa001sjs9vyg40gs2s</t>
+  </si>
+  <si>
+    <t>525U2FII</t>
+  </si>
+  <si>
+    <t>cmvbyb0a8001njs9vz8pz8qii</t>
+  </si>
+  <si>
+    <t>MTBW29SD</t>
+  </si>
+  <si>
+    <t>cmvbyb0a6001ijs9vdohs3i8s</t>
+  </si>
+  <si>
+    <t>LV7LPGAB</t>
+  </si>
+  <si>
+    <t>cmvbyb0a4001djs9vi8uj88wd</t>
+  </si>
+  <si>
+    <t>4S5GGMLY</t>
+  </si>
+  <si>
+    <t>cmvbyb0a10018js9vb432bx4v</t>
+  </si>
+  <si>
+    <t>ITLWWQTR</t>
+  </si>
+  <si>
+    <t>cmvbyb09z0013js9vhv3nhset</t>
+  </si>
+  <si>
+    <t>TP6BHOTS</t>
+  </si>
+  <si>
+    <t>cmvbyb09w000yjs9v36lysqa6</t>
+  </si>
+  <si>
+    <t>THTJ8LNN</t>
+  </si>
+  <si>
+    <t>cmvbyb09t000tjs9vmlv1azmv</t>
+  </si>
+  <si>
+    <t>5GG0KMMS</t>
+  </si>
+  <si>
+    <t>cmvbyb09r000ojs9v2lxqssdl</t>
+  </si>
+  <si>
+    <t>JV08P0L3</t>
+  </si>
+  <si>
+    <t>cmvbyb09p000jjs9vv3kabyrx</t>
+  </si>
+  <si>
+    <t>ZEOXBZYD</t>
+  </si>
+  <si>
+    <t>cmvbyb09m000ejs9vztwmzvyj</t>
+  </si>
+  <si>
+    <t>35ZXBAUP</t>
   </si>
   <si>
     <t>Категория</t>
@@ -455,94 +455,94 @@
     <t>obligation</t>
   </si>
   <si>
-    <t>Заказ gbr7y34t</t>
-  </si>
-  <si>
-    <t>Заказ j6g0jwf5</t>
-  </si>
-  <si>
-    <t>Заказ 4zq8oie0</t>
-  </si>
-  <si>
-    <t>Заказ iyfkyppc</t>
-  </si>
-  <si>
-    <t>Заказ ruvum57v</t>
-  </si>
-  <si>
-    <t>Заказ i91hv26o</t>
-  </si>
-  <si>
-    <t>Заказ c003x63k</t>
-  </si>
-  <si>
-    <t>Заказ nrim4ddm</t>
-  </si>
-  <si>
-    <t>Заказ azi2ffwr</t>
-  </si>
-  <si>
-    <t>Заказ vyllqwja</t>
-  </si>
-  <si>
-    <t>Заказ gskkpbv4</t>
-  </si>
-  <si>
-    <t>Заказ dd9j27oc</t>
-  </si>
-  <si>
-    <t>Заказ s8dtrbn4</t>
-  </si>
-  <si>
-    <t>Заказ yo4ksy06</t>
-  </si>
-  <si>
-    <t>Заказ bydp2289</t>
-  </si>
-  <si>
-    <t>Заказ iv7dln0w</t>
-  </si>
-  <si>
-    <t>Заказ zqy7e814</t>
-  </si>
-  <si>
-    <t>Заказ zyfjtvpo</t>
-  </si>
-  <si>
-    <t>Заказ 3ioqurhf</t>
-  </si>
-  <si>
-    <t>Заказ s1f6ocfw</t>
-  </si>
-  <si>
-    <t>Заказ n585f69r</t>
-  </si>
-  <si>
-    <t>Заказ e1ocdfgb</t>
-  </si>
-  <si>
-    <t>Заказ csdahvhl</t>
-  </si>
-  <si>
-    <t>Заказ hp4ejqwh</t>
-  </si>
-  <si>
-    <t>Заказ 34hou3gn</t>
-  </si>
-  <si>
-    <t>Заказ p0npj3q7</t>
-  </si>
-  <si>
-    <t>Заказ 0o7anaco</t>
-  </si>
-  <si>
-    <t>Заказ wubjhwhv</t>
-  </si>
-  <si>
-    <t>Заказ lz574148</t>
-  </si>
-  <si>
-    <t>Заказ a6oez1t0</t>
+    <t>Заказ lc03kgbt</t>
+  </si>
+  <si>
+    <t>Заказ lkdxm8ow</t>
+  </si>
+  <si>
+    <t>Заказ cjbrhpfj</t>
+  </si>
+  <si>
+    <t>Заказ qiuzezgg</t>
+  </si>
+  <si>
+    <t>Заказ bhcm05ek</t>
+  </si>
+  <si>
+    <t>Заказ p9m18ft2</t>
+  </si>
+  <si>
+    <t>Заказ 6c6gl77t</t>
+  </si>
+  <si>
+    <t>Заказ 47cwr076</t>
+  </si>
+  <si>
+    <t>Заказ u92ykavk</t>
+  </si>
+  <si>
+    <t>Заказ uus4995x</t>
+  </si>
+  <si>
+    <t>Заказ vd41za8k</t>
+  </si>
+  <si>
+    <t>Заказ 0l45acg7</t>
+  </si>
+  <si>
+    <t>Заказ sv8u2sa1</t>
+  </si>
+  <si>
+    <t>Заказ 0ivhrg2h</t>
+  </si>
+  <si>
+    <t>Заказ 17us3xju</t>
+  </si>
+  <si>
+    <t>Заказ cmuyo8ii</t>
+  </si>
+  <si>
+    <t>Заказ uiv2jdsd</t>
+  </si>
+  <si>
+    <t>Заказ dol9hiv8</t>
+  </si>
+  <si>
+    <t>Заказ 1abwouqs</t>
+  </si>
+  <si>
+    <t>Заказ 525u2fii</t>
+  </si>
+  <si>
+    <t>Заказ mtbw29sd</t>
+  </si>
+  <si>
+    <t>Заказ lv7lpgab</t>
+  </si>
+  <si>
+    <t>Заказ 4s5ggmly</t>
+  </si>
+  <si>
+    <t>Заказ itlwwqtr</t>
+  </si>
+  <si>
+    <t>Заказ tp6bhots</t>
+  </si>
+  <si>
+    <t>Заказ thtj8lnn</t>
+  </si>
+  <si>
+    <t>Заказ 5gg0kmms</t>
+  </si>
+  <si>
+    <t>Заказ jv08p0l3</t>
+  </si>
+  <si>
+    <t>Заказ zeoxbzyd</t>
+  </si>
+  <si>
+    <t>Заказ 35zxbaup</t>
   </si>
 </sst>
 </file>

</xml_diff>